<commit_message>
Security remediation and verified retest reports
</commit_message>
<xml_diff>
--- a/Vulnerability Test Results/endpoint-inventory.xlsx
+++ b/Vulnerability Test Results/endpoint-inventory.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="49">
   <si>
     <t>Endpoint</t>
   </si>
@@ -31,16 +31,19 @@
     <t>Authenticated?</t>
   </si>
   <si>
+    <t>Rate Limited?</t>
+  </si>
+  <si>
     <t>/api/auth/login</t>
   </si>
   <si>
     <t>POST</t>
   </si>
   <si>
-    <t>User login lookup</t>
-  </si>
-  <si>
-    <t>email</t>
+    <t>User authentication &amp; JWT issue</t>
+  </si>
+  <si>
+    <t>email, password</t>
   </si>
   <si>
     <t>Any</t>
@@ -49,13 +52,16 @@
     <t>No</t>
   </si>
   <si>
+    <t>Yes (20/15min)</t>
+  </si>
+  <si>
     <t>/api/auth/register</t>
   </si>
   <si>
-    <t>Create user account</t>
-  </si>
-  <si>
-    <t>name, email, department, role, rollNumber, phone</t>
+    <t>Create new user account</t>
+  </si>
+  <si>
+    <t>name, email, password, role, department, rollNumber, phone</t>
   </si>
   <si>
     <t>/api/auth/profile</t>
@@ -67,7 +73,16 @@
     <t>Update profile properties</t>
   </si>
   <si>
-    <t>userId, phone, etc.</t>
+    <t>userId, phone, department</t>
+  </si>
+  <si>
+    <t>Authenticated User</t>
+  </si>
+  <si>
+    <t>Yes (JWT)</t>
+  </si>
+  <si>
+    <t>Yes (200/15min)</t>
   </si>
   <si>
     <t>/api/events</t>
@@ -82,18 +97,15 @@
     <t>None</t>
   </si>
   <si>
-    <t>Create new event details</t>
-  </si>
-  <si>
-    <t>title, host, date, etc.</t>
+    <t>Publish new event</t>
+  </si>
+  <si>
+    <t>title, description, category, date, venue, capacity</t>
   </si>
   <si>
     <t>ADMIN, FACULTY</t>
   </si>
   <si>
-    <t>No (Backend missing check)</t>
-  </si>
-  <si>
     <t>/api/events/:id</t>
   </si>
   <si>
@@ -106,7 +118,7 @@
     <t>Update event metadata</t>
   </si>
   <si>
-    <t>id, title, etc.</t>
+    <t>id, title, venue, etc.</t>
   </si>
   <si>
     <t>DELETE</t>
@@ -121,10 +133,10 @@
     <t>/api/events/:id/register</t>
   </si>
   <si>
-    <t>Register user to event</t>
-  </si>
-  <si>
-    <t>id, userId, userName, etc.</t>
+    <t>Register user for event</t>
+  </si>
+  <si>
+    <t>id, name, email, roll</t>
   </si>
   <si>
     <t>/api/events/:id/register/:userId</t>
@@ -140,6 +152,12 @@
   </si>
   <si>
     <t>Mark attendee attendance</t>
+  </si>
+  <si>
+    <t>/api/health</t>
+  </si>
+  <si>
+    <t>Health check &amp; security header test</t>
   </si>
 </sst>
 </file>
@@ -526,7 +544,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -534,10 +552,10 @@
     <col min="3" max="3" width="45" customWidth="1"/>
     <col min="4" max="4" width="25" customWidth="1"/>
     <col min="5" max="5" width="20" customWidth="1"/>
-    <col min="6" max="6" width="15" customWidth="1"/>
+    <col min="6" max="7" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -556,225 +574,284 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" t="s">
         <v>8</v>
       </c>
-      <c r="D2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F2" t="s">
+      <c r="C3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="F3" t="s">
         <v>12</v>
       </c>
-      <c r="B3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="G3" t="s">
         <v>13</v>
       </c>
-      <c r="D3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" t="s">
-        <v>10</v>
-      </c>
-      <c r="F3" t="s">
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" t="s">
+        <v>22</v>
+      </c>
+      <c r="G4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C4" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4" t="s">
+      <c r="F5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" t="s">
+        <v>29</v>
+      </c>
+      <c r="E6" t="s">
+        <v>30</v>
+      </c>
+      <c r="F6" t="s">
+        <v>22</v>
+      </c>
+      <c r="G6" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" t="s">
+        <v>32</v>
+      </c>
+      <c r="D7" t="s">
+        <v>33</v>
+      </c>
+      <c r="E7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" t="s">
+        <v>12</v>
+      </c>
+      <c r="G7" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>31</v>
+      </c>
+      <c r="B8" t="s">
         <v>18</v>
       </c>
-      <c r="E4" t="s">
-        <v>10</v>
-      </c>
-      <c r="F4" t="s">
+      <c r="C8" t="s">
+        <v>34</v>
+      </c>
+      <c r="D8" t="s">
+        <v>35</v>
+      </c>
+      <c r="E8" t="s">
+        <v>30</v>
+      </c>
+      <c r="F8" t="s">
+        <v>22</v>
+      </c>
+      <c r="G8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9" t="s">
+        <v>37</v>
+      </c>
+      <c r="D9" t="s">
+        <v>33</v>
+      </c>
+      <c r="E9" t="s">
+        <v>38</v>
+      </c>
+      <c r="F9" t="s">
+        <v>22</v>
+      </c>
+      <c r="G9" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>39</v>
+      </c>
+      <c r="B10" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" t="s">
+        <v>40</v>
+      </c>
+      <c r="D10" t="s">
+        <v>41</v>
+      </c>
+      <c r="E10" t="s">
+        <v>21</v>
+      </c>
+      <c r="F10" t="s">
+        <v>22</v>
+      </c>
+      <c r="G10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>42</v>
+      </c>
+      <c r="B11" t="s">
+        <v>36</v>
+      </c>
+      <c r="C11" t="s">
+        <v>43</v>
+      </c>
+      <c r="D11" t="s">
+        <v>44</v>
+      </c>
+      <c r="E11" t="s">
+        <v>21</v>
+      </c>
+      <c r="F11" t="s">
+        <v>22</v>
+      </c>
+      <c r="G11" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>45</v>
+      </c>
+      <c r="B12" t="s">
+        <v>8</v>
+      </c>
+      <c r="C12" t="s">
+        <v>46</v>
+      </c>
+      <c r="D12" t="s">
+        <v>44</v>
+      </c>
+      <c r="E12" t="s">
+        <v>30</v>
+      </c>
+      <c r="F12" t="s">
+        <v>22</v>
+      </c>
+      <c r="G12" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>47</v>
+      </c>
+      <c r="B13" t="s">
+        <v>25</v>
+      </c>
+      <c r="C13" t="s">
+        <v>48</v>
+      </c>
+      <c r="D13" t="s">
+        <v>27</v>
+      </c>
+      <c r="E13" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C5" t="s">
-        <v>21</v>
-      </c>
-      <c r="D5" t="s">
-        <v>22</v>
-      </c>
-      <c r="E5" t="s">
-        <v>10</v>
-      </c>
-      <c r="F5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>19</v>
-      </c>
-      <c r="B6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C6" t="s">
-        <v>23</v>
-      </c>
-      <c r="D6" t="s">
-        <v>24</v>
-      </c>
-      <c r="E6" t="s">
-        <v>25</v>
-      </c>
-      <c r="F6" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>27</v>
-      </c>
-      <c r="B7" t="s">
-        <v>20</v>
-      </c>
-      <c r="C7" t="s">
-        <v>28</v>
-      </c>
-      <c r="D7" t="s">
-        <v>29</v>
-      </c>
-      <c r="E7" t="s">
-        <v>10</v>
-      </c>
-      <c r="F7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>27</v>
-      </c>
-      <c r="B8" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" t="s">
-        <v>30</v>
-      </c>
-      <c r="D8" t="s">
-        <v>31</v>
-      </c>
-      <c r="E8" t="s">
-        <v>25</v>
-      </c>
-      <c r="F8" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>27</v>
-      </c>
-      <c r="B9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C9" t="s">
-        <v>33</v>
-      </c>
-      <c r="D9" t="s">
-        <v>29</v>
-      </c>
-      <c r="E9" t="s">
-        <v>34</v>
-      </c>
-      <c r="F9" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>35</v>
-      </c>
-      <c r="B10" t="s">
-        <v>7</v>
-      </c>
-      <c r="C10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D10" t="s">
-        <v>37</v>
-      </c>
-      <c r="E10" t="s">
-        <v>10</v>
-      </c>
-      <c r="F10" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>38</v>
-      </c>
-      <c r="B11" t="s">
-        <v>32</v>
-      </c>
-      <c r="C11" t="s">
-        <v>39</v>
-      </c>
-      <c r="D11" t="s">
-        <v>40</v>
-      </c>
-      <c r="E11" t="s">
-        <v>10</v>
-      </c>
-      <c r="F11" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>41</v>
-      </c>
-      <c r="B12" t="s">
-        <v>7</v>
-      </c>
-      <c r="C12" t="s">
-        <v>42</v>
-      </c>
-      <c r="D12" t="s">
-        <v>40</v>
-      </c>
-      <c r="E12" t="s">
-        <v>25</v>
-      </c>
-      <c r="F12" t="s">
-        <v>11</v>
+      <c r="F13" t="s">
+        <v>12</v>
+      </c>
+      <c r="G13" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>